<commit_message>
Excel-Export nach Großvater-Zahlung aktualisieren
</commit_message>
<xml_diff>
--- a/exports/Urlaubskasse_Woche1.xlsx
+++ b/exports/Urlaubskasse_Woche1.xlsx
@@ -2,17 +2,120 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R9baede98870b4966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R10bb9d0ff2a84198"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="R32e784a1fd274433"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zahlungen" sheetId="4" r:id="R766ecbda2390422e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salden" sheetId="5" r:id="R775eb1ea158f4860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="Rbdc5394ee54b4447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R260515aa54b944ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="R42fe89670cb14239"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zahlungen" sheetId="4" r:id="R06dea000f8a44900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salden" sheetId="5" r:id="R2920caad5d9944e0"/>
   </x:sheets>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="#,##0.00 [$€-de-DE]"/>
+  </x:numFmts>
+  <x:fonts count="4">
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF173F37"/>
+      <x:name val="Carlito"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="4">
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173F37"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCEAE5"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="2">
+    <x:border/>
+    <x:border/>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="19">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0"/>
+  </x:cellStyles>
+  <x:dxfs count="2">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF167A5B"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA3473D"/>
+      </x:font>
+    </x:dxf>
+  </x:dxfs>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -215,7 +318,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="F4" s="8" t="n">
-        <x:v>83.16</x:v>
+        <x:v>87.16</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -232,7 +335,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="F5" s="8" t="n">
-        <x:v>26.9</x:v>
+        <x:v>30.9</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -240,7 +343,7 @@
         <x:v>Verrechnete Ausgaben</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>703.02</x:v>
+        <x:v>719.02</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Tante</x:v>
@@ -249,7 +352,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="F6" s="8" t="n">
-        <x:v>168.57</x:v>
+        <x:v>156.57</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -257,7 +360,16 @@
         <x:v>Beleg-/Ausgabensumme</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>760.99</x:v>
+        <x:v>776.99</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Tante</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Großvater</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="n">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -369,6 +481,29 @@
       </x:c>
       <x:c r="G15" t="str">
         <x:v>AUS-20260721-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>21.07.2026</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Bezahlung Großvater</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>Großvater</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>ohne Bon</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>AUS-20260721-002</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -738,6 +873,29 @@
         <x:v>Onkel</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>AUS-20260721-002</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>21.07.2026</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Bezahlung Großvater</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="E16" s="8" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F16" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Großvater</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -986,6 +1144,29 @@
         <x:v>8.75</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>AUS-20260721-002</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1229,6 +1410,17 @@
       </x:c>
       <x:c r="C21" s="8" t="n">
         <x:v>35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>AUS-20260721-002</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>Großvater</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="n">
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1265,13 +1457,13 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="B2" s="8" t="n">
-        <x:v>166.13</x:v>
+        <x:v>170.13</x:v>
       </x:c>
       <x:c r="C2" s="8" t="n">
         <x:v>444.76</x:v>
       </x:c>
       <x:c r="D2" s="8" t="n">
-        <x:v>278.63</x:v>
+        <x:v>274.63</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1279,13 +1471,13 @@
         <x:v>Katrin</x:v>
       </x:c>
       <x:c r="B3" s="8" t="n">
-        <x:v>199.72</x:v>
+        <x:v>203.72</x:v>
       </x:c>
       <x:c r="C3" s="8" t="n">
         <x:v>116.56</x:v>
       </x:c>
       <x:c r="D3" s="8" t="n">
-        <x:v>-83.16</x:v>
+        <x:v>-87.16</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1293,13 +1485,13 @@
         <x:v>Onkel</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>168.6</x:v>
+        <x:v>172.6</x:v>
       </x:c>
       <x:c r="C4" s="8" t="n">
         <x:v>141.7</x:v>
       </x:c>
       <x:c r="D4" s="8" t="n">
-        <x:v>-26.9</x:v>
+        <x:v>-30.9</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1307,13 +1499,13 @@
         <x:v>Tante</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>168.57</x:v>
+        <x:v>172.57</x:v>
       </x:c>
       <x:c r="C5" s="8" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="8" t="n">
-        <x:v>-168.57</x:v>
+        <x:v>-172.57</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1338,10 +1530,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D7" s="8" t="n">
-        <x:v>0</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Excel-Export nach Frischemarkt und Tierpark aktualisieren
</commit_message>
<xml_diff>
--- a/exports/Urlaubskasse_Woche1.xlsx
+++ b/exports/Urlaubskasse_Woche1.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="Rbdc5394ee54b4447"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R260515aa54b944ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="R42fe89670cb14239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zahlungen" sheetId="4" r:id="R06dea000f8a44900"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salden" sheetId="5" r:id="R2920caad5d9944e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R989babc36b694c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R1ef8215cfe104de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="R0318212ec5ae490f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zahlungen" sheetId="4" r:id="R05f428fbd5e04303"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salden" sheetId="5" r:id="R94db848dee51420a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -318,7 +318,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="F4" s="8" t="n">
-        <x:v>87.16</x:v>
+        <x:v>106.92</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -335,7 +335,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="F5" s="8" t="n">
-        <x:v>30.9</x:v>
+        <x:v>50.66</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -343,7 +343,7 @@
         <x:v>Verrechnete Ausgaben</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>719.02</x:v>
+        <x:v>798.05</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Tante</x:v>
@@ -352,7 +352,7 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="F6" s="8" t="n">
-        <x:v>156.57</x:v>
+        <x:v>176.32</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -360,7 +360,7 @@
         <x:v>Beleg-/Ausgabensumme</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>776.99</x:v>
+        <x:v>856.02</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Tante</x:v>
@@ -504,6 +504,52 @@
       </x:c>
       <x:c r="G16" t="str">
         <x:v>AUS-20260721-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>23.07.2026</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Frischemarkt Boitzenburg</x:v>
+      </x:c>
+      <x:c r="C17" s="8" t="n">
+        <x:v>59.03</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Foto</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>BON-20260723-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>21.07.2026</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Tierpark Angermünde</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>ohne Bon</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>AUS-20260721-003</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -896,6 +942,52 @@
         <x:v>Großvater</x:v>
       </x:c>
     </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>BON-20260723-001</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>23.07.2026</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Frischemarkt Boitzenburg</x:v>
+      </x:c>
+      <x:c r="D17" s="8" t="n">
+        <x:v>59.03</x:v>
+      </x:c>
+      <x:c r="E17" s="8" t="n">
+        <x:v>59.03</x:v>
+      </x:c>
+      <x:c r="F17" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>AUS-20260721-003</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>21.07.2026</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Tierpark Angermünde</x:v>
+      </x:c>
+      <x:c r="D18" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E18" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F18" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1167,6 +1259,52 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>BON-20260723-001</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+      <x:c r="C12" s="8" t="n">
+        <x:v>59.03</x:v>
+      </x:c>
+      <x:c r="D12" s="8" t="n">
+        <x:v>14.76</x:v>
+      </x:c>
+      <x:c r="E12" s="8" t="n">
+        <x:v>14.76</x:v>
+      </x:c>
+      <x:c r="F12" s="8" t="n">
+        <x:v>14.76</x:v>
+      </x:c>
+      <x:c r="G12" s="8" t="n">
+        <x:v>14.75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>AUS-20260721-003</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Gemeinschaft</x:v>
+      </x:c>
+      <x:c r="C13" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E13" s="8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F13" s="8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G13" s="8" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1421,6 +1559,28 @@
       </x:c>
       <x:c r="C22" s="8" t="n">
         <x:v>16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>BON-20260723-001</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="n">
+        <x:v>59.03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>AUS-20260721-003</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="C24" s="8" t="n">
+        <x:v>20</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1457,13 +1617,13 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="B2" s="8" t="n">
-        <x:v>170.13</x:v>
+        <x:v>189.89</x:v>
       </x:c>
       <x:c r="C2" s="8" t="n">
-        <x:v>444.76</x:v>
+        <x:v>523.79</x:v>
       </x:c>
       <x:c r="D2" s="8" t="n">
-        <x:v>274.63</x:v>
+        <x:v>333.9</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1471,13 +1631,13 @@
         <x:v>Katrin</x:v>
       </x:c>
       <x:c r="B3" s="8" t="n">
-        <x:v>203.72</x:v>
+        <x:v>223.48</x:v>
       </x:c>
       <x:c r="C3" s="8" t="n">
         <x:v>116.56</x:v>
       </x:c>
       <x:c r="D3" s="8" t="n">
-        <x:v>-87.16</x:v>
+        <x:v>-106.92</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1485,13 +1645,13 @@
         <x:v>Onkel</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>172.6</x:v>
+        <x:v>192.36</x:v>
       </x:c>
       <x:c r="C4" s="8" t="n">
         <x:v>141.7</x:v>
       </x:c>
       <x:c r="D4" s="8" t="n">
-        <x:v>-30.9</x:v>
+        <x:v>-50.66</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1499,13 +1659,13 @@
         <x:v>Tante</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>172.57</x:v>
+        <x:v>192.32</x:v>
       </x:c>
       <x:c r="C5" s="8" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="8" t="n">
-        <x:v>-172.57</x:v>
+        <x:v>-192.32</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>

<commit_message>
Excel-Export nach Ponyreiten aktualisieren
</commit_message>
<xml_diff>
--- a/exports/Urlaubskasse_Woche1.xlsx
+++ b/exports/Urlaubskasse_Woche1.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="R06da2ddaccf54905"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R1caf1b584085452f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="R0aa855aef3b34634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zahlungen" sheetId="4" r:id="R21249e4bea2745d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salden" sheetId="5" r:id="R50bf5c19d31f4b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Übersicht" sheetId="1" r:id="Rd5e704ba7b1040c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vorgänge" sheetId="2" r:id="R9bb59df9e80245d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kostenblöcke" sheetId="3" r:id="Reee61fb50db94bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Zahlungen" sheetId="4" r:id="R07f1c17b8d3a4aeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salden" sheetId="5" r:id="R7263292908054179"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -263,350 +263,6 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="14" t="str">
-        <x:v>Urlaubskasse Woche 1</x:v>
-      </x:c>
-      <x:c r="B1" s="14"/>
-      <x:c r="C1" s="14"/>
-      <x:c r="D1" s="14"/>
-      <x:c r="E1" s="14"/>
-      <x:c r="F1" s="14"/>
-      <x:c r="G1" s="14"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="6" t="str">
-        <x:v>Kennzahl</x:v>
-      </x:c>
-      <x:c r="B3" s="6" t="str">
-        <x:v>Wert</x:v>
-      </x:c>
-      <x:c r="D3" s="6" t="str">
-        <x:v>Zahler</x:v>
-      </x:c>
-      <x:c r="E3" s="6" t="str">
-        <x:v>Empfänger</x:v>
-      </x:c>
-      <x:c r="F3" s="6" t="str">
-        <x:v>Betrag</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>Stand</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>21.07.2026</x:v>
-      </x:c>
-      <x:c r="D4" t="str">
-        <x:v>Katrin</x:v>
-      </x:c>
-      <x:c r="E4" t="str">
-        <x:v>Simon</x:v>
-      </x:c>
-      <x:c r="F4" s="8" t="n">
-        <x:v>116.63</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>Woche</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>Woche 1 – offen</x:v>
-      </x:c>
-      <x:c r="D5" t="str">
-        <x:v>Onkel</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>Simon</x:v>
-      </x:c>
-      <x:c r="F5" s="8" t="n">
-        <x:v>21.54</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>Verrechnete Ausgaben</x:v>
-      </x:c>
-      <x:c r="B6" s="8" t="n">
-        <x:v>836.87</x:v>
-      </x:c>
-      <x:c r="D6" t="str">
-        <x:v>Tante</x:v>
-      </x:c>
-      <x:c r="E6" t="str">
-        <x:v>Simon</x:v>
-      </x:c>
-      <x:c r="F6" s="8" t="n">
-        <x:v>186.02</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" t="str">
-        <x:v>Beleg-/Ausgabensumme</x:v>
-      </x:c>
-      <x:c r="B7" s="8" t="n">
-        <x:v>899.24</x:v>
-      </x:c>
-      <x:c r="D7" t="str">
-        <x:v>Tante</x:v>
-      </x:c>
-      <x:c r="E7" t="str">
-        <x:v>Großvater</x:v>
-      </x:c>
-      <x:c r="F7" s="8" t="n">
-        <x:v>16</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" t="str">
-        <x:v>Ausgeschlossen</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="n">
-        <x:v>62.37</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="11" t="str">
-        <x:v>Neu erfasst</x:v>
-      </x:c>
-      <x:c r="B11" s="11"/>
-      <x:c r="C11" s="11"/>
-      <x:c r="D11" s="11"/>
-      <x:c r="E11" s="11"/>
-      <x:c r="F11" s="11"/>
-      <x:c r="G11" s="11"/>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="6" t="str">
-        <x:v>Datum</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="str">
-        <x:v>Händler</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="str">
-        <x:v>Betrag</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="str">
-        <x:v>Verteilung</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="str">
-        <x:v>Bezahlt von</x:v>
-      </x:c>
-      <x:c r="F12" s="6" t="str">
-        <x:v>Beleg</x:v>
-      </x:c>
-      <x:c r="G12" s="6" t="str">
-        <x:v>Vorgang</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>16.07.2026</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>BIO COMPANY Turmstraße</x:v>
-      </x:c>
-      <x:c r="C13" s="8" t="n">
-        <x:v>24.74</x:v>
-      </x:c>
-      <x:c r="D13" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
-        <x:v>Onkel</x:v>
-      </x:c>
-      <x:c r="F13" t="str">
-        <x:v>Foto</x:v>
-      </x:c>
-      <x:c r="G13" t="str">
-        <x:v>BON-20260716-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>16.07.2026</x:v>
-      </x:c>
-      <x:c r="B14" t="str">
-        <x:v>E-Center Berlin-Moabit</x:v>
-      </x:c>
-      <x:c r="C14" s="8" t="n">
-        <x:v>81.96</x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>Onkel</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>Foto</x:v>
-      </x:c>
-      <x:c r="G14" t="str">
-        <x:v>BON-20260716-004</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>21.07.2026</x:v>
-      </x:c>
-      <x:c r="B15" t="str">
-        <x:v>REWE</x:v>
-      </x:c>
-      <x:c r="C15" s="8" t="n">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>Onkel</x:v>
-      </x:c>
-      <x:c r="F15" t="str">
-        <x:v>ohne Bon</x:v>
-      </x:c>
-      <x:c r="G15" t="str">
-        <x:v>AUS-20260721-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="str">
-        <x:v>21.07.2026</x:v>
-      </x:c>
-      <x:c r="B16" t="str">
-        <x:v>Bezahlung Großvater</x:v>
-      </x:c>
-      <x:c r="C16" s="8" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="D16" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E16" t="str">
-        <x:v>Großvater</x:v>
-      </x:c>
-      <x:c r="F16" t="str">
-        <x:v>ohne Bon</x:v>
-      </x:c>
-      <x:c r="G16" t="str">
-        <x:v>AUS-20260721-002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" t="str">
-        <x:v>23.07.2026</x:v>
-      </x:c>
-      <x:c r="B17" t="str">
-        <x:v>Frischemarkt Boitzenburg</x:v>
-      </x:c>
-      <x:c r="C17" s="8" t="n">
-        <x:v>59.03</x:v>
-      </x:c>
-      <x:c r="D17" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E17" t="str">
-        <x:v>Simon</x:v>
-      </x:c>
-      <x:c r="F17" t="str">
-        <x:v>Foto</x:v>
-      </x:c>
-      <x:c r="G17" t="str">
-        <x:v>BON-20260723-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" t="str">
-        <x:v>21.07.2026</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Tierpark Angermünde</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
-        <x:v>Simon</x:v>
-      </x:c>
-      <x:c r="F18" t="str">
-        <x:v>ohne Bon</x:v>
-      </x:c>
-      <x:c r="G18" t="str">
-        <x:v>AUS-20260721-003</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" t="str">
-        <x:v>23.07.2026</x:v>
-      </x:c>
-      <x:c r="B19" t="str">
-        <x:v>Netto Marken-Discount Gramzow</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="n">
-        <x:v>16.44</x:v>
-      </x:c>
-      <x:c r="D19" t="str">
-        <x:v>12,04 € Gemeinschaft; Zeitschrift ausgeschlossen</x:v>
-      </x:c>
-      <x:c r="E19" t="str">
-        <x:v>Onkel</x:v>
-      </x:c>
-      <x:c r="F19" t="str">
-        <x:v>Foto</x:v>
-      </x:c>
-      <x:c r="G19" t="str">
-        <x:v>BON-20260723-002</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>24.07.2026</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>Netto Marken-Discount Gramzow</x:v>
-      </x:c>
-      <x:c r="C20" s="8" t="n">
-        <x:v>26.78</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>Gemeinschaft</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Onkel</x:v>
-      </x:c>
-      <x:c r="F20" t="str">
-        <x:v>Foto; Datum vorläufig</x:v>
-      </x:c>
-      <x:c r="G20" t="str">
-        <x:v>BON-20260724-001</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:G1"/>
-    <x:mergeCell ref="A11:G11"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1078,6 +734,29 @@
       </x:c>
       <x:c r="G20" t="str">
         <x:v>Onkel</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>AUS-20260724-001</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>24.07.2026</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Ponyreiten</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E21" s="8" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="F21" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Simon</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1443,6 +1122,29 @@
         <x:v>6.69</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>AUS-20260724-001</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Ponyreiten – individuelle Verteilung</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="E16" s="8" t="n">
+        <x:v>12.5</x:v>
+      </x:c>
+      <x:c r="F16" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G16" s="8" t="n">
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1741,6 +1443,17 @@
       </x:c>
       <x:c r="C26" s="8" t="n">
         <x:v>26.78</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>AUS-20260724-001</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>Simon</x:v>
+      </x:c>
+      <x:c r="C27" s="8" t="n">
+        <x:v>65</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1777,13 +1490,13 @@
         <x:v>Simon</x:v>
       </x:c>
       <x:c r="B2" s="8" t="n">
-        <x:v>199.6</x:v>
+        <x:v>212.1</x:v>
       </x:c>
       <x:c r="C2" s="8" t="n">
-        <x:v>523.79</x:v>
+        <x:v>588.79</x:v>
       </x:c>
       <x:c r="D2" s="8" t="n">
-        <x:v>324.19</x:v>
+        <x:v>376.69</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1791,13 +1504,13 @@
         <x:v>Katrin</x:v>
       </x:c>
       <x:c r="B3" s="8" t="n">
-        <x:v>233.19</x:v>
+        <x:v>245.69</x:v>
       </x:c>
       <x:c r="C3" s="8" t="n">
         <x:v>116.56</x:v>
       </x:c>
       <x:c r="D3" s="8" t="n">
-        <x:v>-116.63</x:v>
+        <x:v>-129.13</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1805,13 +1518,13 @@
         <x:v>Onkel</x:v>
       </x:c>
       <x:c r="B4" s="8" t="n">
-        <x:v>202.06</x:v>
+        <x:v>222.06</x:v>
       </x:c>
       <x:c r="C4" s="8" t="n">
         <x:v>180.52</x:v>
       </x:c>
       <x:c r="D4" s="8" t="n">
-        <x:v>-21.54</x:v>
+        <x:v>-41.54</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1819,13 +1532,13 @@
         <x:v>Tante</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>202.02</x:v>
+        <x:v>222.02</x:v>
       </x:c>
       <x:c r="C5" s="8" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D5" s="8" t="n">
-        <x:v>-202.02</x:v>
+        <x:v>-222.02</x:v>
       </x:c>
     </x:row>
     <x:row r="6">

</xml_diff>